<commit_message>
Add Porion dedicated model - 1.25mm MRE 86% SDR2mm
</commit_message>
<xml_diff>
--- a/evaluation_output/evaluation_results.xlsx
+++ b/evaluation_output/evaluation_results.xlsx
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6889999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="C2" t="n">
-        <v>0.528</v>
+        <v>0.552</v>
       </c>
       <c r="D2" t="n">
         <v>0.1916999965906143</v>
@@ -461,10 +461,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.745</v>
+        <v>1.699</v>
       </c>
       <c r="C3" t="n">
-        <v>1.055</v>
+        <v>1.02</v>
       </c>
       <c r="D3" t="n">
         <v>0.4169000089168549</v>
@@ -477,10 +477,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.859</v>
+        <v>1.858</v>
       </c>
       <c r="C4" t="n">
-        <v>1.058</v>
+        <v>1.057</v>
       </c>
       <c r="D4" t="n">
         <v>0.08060000091791153</v>
@@ -493,10 +493,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>0.42</v>
+        <v>0.417</v>
       </c>
       <c r="D5" t="n">
         <v>0.1636999994516373</v>
@@ -509,10 +509,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.082</v>
+        <v>1.049</v>
       </c>
       <c r="C6" t="n">
-        <v>0.622</v>
+        <v>0.649</v>
       </c>
       <c r="D6" t="n">
         <v>0.0835999995470047</v>
@@ -525,10 +525,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.016</v>
+        <v>2.002</v>
       </c>
       <c r="C7" t="n">
-        <v>2.693</v>
+        <v>2.697</v>
       </c>
       <c r="D7" t="n">
         <v>0.2822999954223633</v>
@@ -541,10 +541,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.171</v>
+        <v>2.167</v>
       </c>
       <c r="C8" t="n">
-        <v>1.728</v>
+        <v>1.731</v>
       </c>
       <c r="D8" t="n">
         <v>0.09470000118017197</v>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.034</v>
+        <v>1.026</v>
       </c>
       <c r="C9" t="n">
         <v>0.602</v>
@@ -573,10 +573,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.439</v>
+        <v>1.457</v>
       </c>
       <c r="C10" t="n">
-        <v>0.776</v>
+        <v>0.79</v>
       </c>
       <c r="D10" t="n">
         <v>0.08179999887943268</v>
@@ -589,10 +589,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.795</v>
+        <v>0.782</v>
       </c>
       <c r="C11" t="n">
-        <v>0.629</v>
+        <v>0.614</v>
       </c>
       <c r="D11" t="n">
         <v>0.1581999957561493</v>
@@ -605,10 +605,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3.055</v>
+        <v>3.046</v>
       </c>
       <c r="C12" t="n">
-        <v>3.217</v>
+        <v>3.222</v>
       </c>
       <c r="D12" t="n">
         <v>0.08860000222921371</v>
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.462</v>
+        <v>1.446</v>
       </c>
       <c r="C13" t="n">
-        <v>1.503</v>
+        <v>1.446</v>
       </c>
       <c r="D13" t="n">
         <v>0.323500007390976</v>
@@ -637,10 +637,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.924</v>
+        <v>0.989</v>
       </c>
       <c r="C14" t="n">
-        <v>0.577</v>
+        <v>0.783</v>
       </c>
       <c r="D14" t="n">
         <v>0.08730000257492065</v>
@@ -653,10 +653,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.311</v>
+        <v>0.95</v>
       </c>
       <c r="C15" t="n">
-        <v>1.767</v>
+        <v>0.433</v>
       </c>
       <c r="D15" t="n">
         <v>0.1890999972820282</v>
@@ -669,10 +669,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.146</v>
+        <v>1.068</v>
       </c>
       <c r="C16" t="n">
-        <v>0.841</v>
+        <v>0.845</v>
       </c>
       <c r="D16" t="n">
         <v>0.0917000025510788</v>
@@ -685,10 +685,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.739</v>
+        <v>0.804</v>
       </c>
       <c r="C17" t="n">
-        <v>0.327</v>
+        <v>0.44</v>
       </c>
       <c r="D17" t="n">
         <v>0.2691999971866608</v>
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.876</v>
+        <v>1.903</v>
       </c>
       <c r="C18" t="n">
-        <v>2.144</v>
+        <v>2.261</v>
       </c>
       <c r="D18" t="n">
         <v>0.08380000293254852</v>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.548</v>
+        <v>0.521</v>
       </c>
       <c r="C19" t="n">
-        <v>0.351</v>
+        <v>0.358</v>
       </c>
       <c r="D19" t="n">
         <v>0.193000003695488</v>
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.008</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="C21" t="n">
-        <v>1.838</v>
+        <v>1.551</v>
       </c>
       <c r="D21" t="n">
         <v>0.1849000006914139</v>
@@ -765,10 +765,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2.113</v>
+        <v>2.11</v>
       </c>
       <c r="C22" t="n">
-        <v>2.3</v>
+        <v>2.288</v>
       </c>
       <c r="D22" t="n">
         <v>0.08209999650716782</v>
@@ -781,10 +781,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.074</v>
+        <v>1.118</v>
       </c>
       <c r="C23" t="n">
-        <v>0.587</v>
+        <v>0.706</v>
       </c>
       <c r="D23" t="n">
         <v>0.3461999893188477</v>
@@ -797,10 +797,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.209</v>
+        <v>1.207</v>
       </c>
       <c r="C24" t="n">
-        <v>1.05</v>
+        <v>1.051</v>
       </c>
       <c r="D24" t="n">
         <v>0.2806000113487244</v>
@@ -813,10 +813,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1.047</v>
+        <v>1.059</v>
       </c>
       <c r="C25" t="n">
-        <v>0.442</v>
+        <v>0.446</v>
       </c>
       <c r="D25" t="n">
         <v>0.1905999928712845</v>
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1.17</v>
+        <v>1.127</v>
       </c>
       <c r="C26" t="n">
-        <v>1.207</v>
+        <v>1.171</v>
       </c>
       <c r="D26" t="n">
         <v>0.08349999785423279</v>
@@ -845,10 +845,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1.218</v>
+        <v>1.184</v>
       </c>
       <c r="C27" t="n">
-        <v>0.447</v>
+        <v>0.443</v>
       </c>
       <c r="D27" t="n">
         <v>0.4440000057220459</v>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1.139</v>
+        <v>1.162</v>
       </c>
       <c r="C28" t="n">
         <v>0.767</v>
@@ -877,10 +877,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.997</v>
+        <v>0.886</v>
       </c>
       <c r="C29" t="n">
-        <v>0.839</v>
+        <v>0.485</v>
       </c>
       <c r="D29" t="n">
         <v>0.2987000048160553</v>
@@ -893,10 +893,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.682</v>
+        <v>1.732</v>
       </c>
       <c r="C30" t="n">
-        <v>1.385</v>
+        <v>1.382</v>
       </c>
       <c r="D30" t="n">
         <v>0.07599999755620956</v>
@@ -909,10 +909,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.702</v>
+        <v>0.742</v>
       </c>
       <c r="C31" t="n">
-        <v>0.549</v>
+        <v>0.609</v>
       </c>
       <c r="D31" t="n">
         <v>0.1624000072479248</v>
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.632</v>
+        <v>1.618</v>
       </c>
       <c r="C32" t="n">
-        <v>0.928</v>
+        <v>0.915</v>
       </c>
       <c r="D32" t="n">
         <v>0.08020000159740448</v>
@@ -941,10 +941,10 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1.255</v>
+        <v>1.312</v>
       </c>
       <c r="C33" t="n">
-        <v>0.866</v>
+        <v>0.854</v>
       </c>
       <c r="D33" t="n">
         <v>0.1343999952077866</v>
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.555</v>
+        <v>1.487</v>
       </c>
       <c r="C34" t="n">
-        <v>0.821</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="D34" t="n">
         <v>0.08030000329017639</v>
@@ -973,10 +973,10 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1.169</v>
+        <v>1.134</v>
       </c>
       <c r="C35" t="n">
-        <v>0.598</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="D35" t="n">
         <v>0.1518000066280365</v>
@@ -989,10 +989,10 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.957</v>
+        <v>0.886</v>
       </c>
       <c r="C36" t="n">
-        <v>0.896</v>
+        <v>0.773</v>
       </c>
       <c r="D36" t="n">
         <v>0.07620000094175339</v>
@@ -1005,10 +1005,10 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.886</v>
+        <v>0.968</v>
       </c>
       <c r="C37" t="n">
-        <v>0.705</v>
+        <v>0.704</v>
       </c>
       <c r="D37" t="n">
         <v>0.2922999858856201</v>
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.948</v>
       </c>
       <c r="C38" t="n">
-        <v>0.681</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="D38" t="n">
         <v>0.07890000194311142</v>
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.954</v>
+        <v>1.022</v>
       </c>
       <c r="C39" t="n">
-        <v>0.412</v>
+        <v>0.451</v>
       </c>
       <c r="D39" t="n">
         <v>0.1588999927043915</v>
@@ -1053,10 +1053,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.957</v>
+        <v>0.961</v>
       </c>
       <c r="C40" t="n">
-        <v>0.47</v>
+        <v>0.468</v>
       </c>
       <c r="D40" t="n">
         <v>0.2276999950408936</v>
@@ -1085,10 +1085,10 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1.128</v>
+        <v>1.136</v>
       </c>
       <c r="C42" t="n">
-        <v>0.594</v>
+        <v>0.605</v>
       </c>
       <c r="D42" t="n">
         <v>0.08229999989271164</v>
@@ -1101,10 +1101,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.211</v>
+        <v>1.166</v>
       </c>
       <c r="C43" t="n">
-        <v>0.654</v>
+        <v>0.629</v>
       </c>
       <c r="D43" t="n">
         <v>0.1342000067234039</v>
@@ -1117,10 +1117,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1.135</v>
+        <v>1.15</v>
       </c>
       <c r="C44" t="n">
-        <v>0.865</v>
+        <v>0.871</v>
       </c>
       <c r="D44" t="n">
         <v>0.08209999650716782</v>
@@ -1133,10 +1133,10 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1.112</v>
+        <v>1.008</v>
       </c>
       <c r="C45" t="n">
-        <v>0.792</v>
+        <v>0.58</v>
       </c>
       <c r="D45" t="n">
         <v>0.1850000023841858</v>
@@ -1149,10 +1149,10 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1.654</v>
+        <v>1.841</v>
       </c>
       <c r="C46" t="n">
-        <v>1.183</v>
+        <v>1.81</v>
       </c>
       <c r="D46" t="n">
         <v>0.2212000042200089</v>
@@ -1165,10 +1165,10 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1.031</v>
+        <v>0.988</v>
       </c>
       <c r="C47" t="n">
-        <v>0.454</v>
+        <v>0.482</v>
       </c>
       <c r="D47" t="n">
         <v>0.2096000015735626</v>
@@ -1181,10 +1181,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.59</v>
+        <v>1.539</v>
       </c>
       <c r="C48" t="n">
-        <v>1.231</v>
+        <v>1.189</v>
       </c>
       <c r="D48" t="n">
         <v>0.08209999650716782</v>
@@ -1197,10 +1197,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1.116</v>
+        <v>1.094</v>
       </c>
       <c r="C49" t="n">
-        <v>1.788</v>
+        <v>1.69</v>
       </c>
       <c r="D49" t="n">
         <v>0.1492999941110611</v>
@@ -1213,10 +1213,10 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1.306</v>
+        <v>1.295</v>
       </c>
       <c r="C50" t="n">
-        <v>0.921</v>
+        <v>0.879</v>
       </c>
       <c r="D50" t="n">
         <v>0.08389999717473984</v>
@@ -1229,10 +1229,10 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.527</v>
+        <v>0.538</v>
       </c>
       <c r="C51" t="n">
-        <v>0.441</v>
+        <v>0.48</v>
       </c>
       <c r="D51" t="n">
         <v>0.2011999934911728</v>
@@ -1245,10 +1245,10 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1.698</v>
+        <v>1.707</v>
       </c>
       <c r="C52" t="n">
-        <v>1.281</v>
+        <v>1.288</v>
       </c>
       <c r="D52" t="n">
         <v>0.08649999648332596</v>
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.697</v>
+        <v>0.72</v>
       </c>
       <c r="C53" t="n">
-        <v>0.306</v>
+        <v>0.325</v>
       </c>
       <c r="D53" t="n">
         <v>0.2937999963760376</v>
@@ -1277,10 +1277,10 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.892</v>
       </c>
       <c r="C54" t="n">
-        <v>0.504</v>
+        <v>0.473</v>
       </c>
       <c r="D54" t="n">
         <v>0.08219999819993973</v>
@@ -1293,10 +1293,10 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1.557</v>
+        <v>1.517</v>
       </c>
       <c r="C55" t="n">
-        <v>2.069</v>
+        <v>1.895</v>
       </c>
       <c r="D55" t="n">
         <v>0.2419999986886978</v>
@@ -1309,10 +1309,10 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.629</v>
+        <v>0.601</v>
       </c>
       <c r="C56" t="n">
-        <v>0.309</v>
+        <v>0.291</v>
       </c>
       <c r="D56" t="n">
         <v>0.1372999995946884</v>
@@ -1325,10 +1325,10 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1.522</v>
+        <v>1.567</v>
       </c>
       <c r="C57" t="n">
-        <v>1.743</v>
+        <v>1.744</v>
       </c>
       <c r="D57" t="n">
         <v>0.197500005364418</v>
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1.433</v>
+        <v>1.427</v>
       </c>
       <c r="C58" t="n">
-        <v>1.617</v>
+        <v>1.618</v>
       </c>
       <c r="D58" t="n">
         <v>0.1391000002622604</v>
@@ -1357,10 +1357,10 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.98</v>
+        <v>0.869</v>
       </c>
       <c r="C59" t="n">
-        <v>0.793</v>
+        <v>0.681</v>
       </c>
       <c r="D59" t="n">
         <v>0.1955000013113022</v>
@@ -1373,10 +1373,10 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1.255</v>
+        <v>1.218</v>
       </c>
       <c r="C60" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="D60" t="n">
         <v>0.1343999952077866</v>
@@ -1389,10 +1389,10 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1.129</v>
+        <v>1.134</v>
       </c>
       <c r="C61" t="n">
-        <v>2.108</v>
+        <v>2.13</v>
       </c>
       <c r="D61" t="n">
         <v>0.1588999927043915</v>
@@ -1405,10 +1405,10 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1.331</v>
+        <v>1.264</v>
       </c>
       <c r="C62" t="n">
-        <v>1.113</v>
+        <v>1.102</v>
       </c>
       <c r="D62" t="n">
         <v>0.1303000003099442</v>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.975</v>
+        <v>0.962</v>
       </c>
       <c r="C63" t="n">
         <v>0.402</v>
@@ -1437,10 +1437,10 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1.543</v>
+        <v>1.511</v>
       </c>
       <c r="C64" t="n">
-        <v>0.844</v>
+        <v>0.851</v>
       </c>
       <c r="D64" t="n">
         <v>0.1456999927759171</v>
@@ -1453,10 +1453,10 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.794</v>
+        <v>0.791</v>
       </c>
       <c r="C65" t="n">
-        <v>0.491</v>
+        <v>0.49</v>
       </c>
       <c r="D65" t="n">
         <v>0.1724999994039536</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1.268</v>
+        <v>1.27</v>
       </c>
       <c r="C66" t="n">
         <v>0.619</v>
@@ -1485,10 +1485,10 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1.785</v>
+        <v>1.741</v>
       </c>
       <c r="C67" t="n">
-        <v>0.822</v>
+        <v>0.774</v>
       </c>
       <c r="D67" t="n">
         <v>0.2062000036239624</v>
@@ -1501,10 +1501,10 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1.376</v>
+        <v>1.45</v>
       </c>
       <c r="C68" t="n">
-        <v>1.379</v>
+        <v>1.645</v>
       </c>
       <c r="D68" t="n">
         <v>0.301499992609024</v>
@@ -1517,10 +1517,10 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.829</v>
       </c>
       <c r="C69" t="n">
-        <v>0.452</v>
+        <v>0.451</v>
       </c>
       <c r="D69" t="n">
         <v>0.323199987411499</v>
@@ -1533,10 +1533,10 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1.739</v>
+        <v>1.725</v>
       </c>
       <c r="C70" t="n">
-        <v>1.195</v>
+        <v>1.189</v>
       </c>
       <c r="D70" t="n">
         <v>0.1421999931335449</v>
@@ -1549,10 +1549,10 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.859</v>
+        <v>0.829</v>
       </c>
       <c r="C71" t="n">
-        <v>0.355</v>
+        <v>0.358</v>
       </c>
       <c r="D71" t="n">
         <v>0.2930000126361847</v>
@@ -1565,10 +1565,10 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2.045</v>
+        <v>1.971</v>
       </c>
       <c r="C72" t="n">
-        <v>1.675</v>
+        <v>1.7</v>
       </c>
       <c r="D72" t="n">
         <v>0.1310999989509583</v>
@@ -1581,10 +1581,10 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.961</v>
+        <v>1.059</v>
       </c>
       <c r="C73" t="n">
-        <v>0.805</v>
+        <v>0.876</v>
       </c>
       <c r="D73" t="n">
         <v>0.3048999905586243</v>
@@ -1597,10 +1597,10 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1.806</v>
+        <v>1.717</v>
       </c>
       <c r="C74" t="n">
-        <v>1.06</v>
+        <v>1</v>
       </c>
       <c r="D74" t="n">
         <v>0.1424999982118607</v>
@@ -1613,10 +1613,10 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.741</v>
+        <v>0.701</v>
       </c>
       <c r="C75" t="n">
-        <v>0.472</v>
+        <v>0.4</v>
       </c>
       <c r="D75" t="n">
         <v>0.4350999891757965</v>
@@ -1629,10 +1629,10 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1.27</v>
+        <v>1.288</v>
       </c>
       <c r="C76" t="n">
-        <v>0.625</v>
+        <v>0.628</v>
       </c>
       <c r="D76" t="n">
         <v>0.1506000012159348</v>
@@ -1645,10 +1645,10 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.778</v>
+        <v>0.805</v>
       </c>
       <c r="C77" t="n">
-        <v>0.88</v>
+        <v>0.872</v>
       </c>
       <c r="D77" t="n">
         <v>0.2311999946832657</v>
@@ -1661,10 +1661,10 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1.303</v>
+        <v>1.286</v>
       </c>
       <c r="C78" t="n">
-        <v>0.742</v>
+        <v>0.747</v>
       </c>
       <c r="D78" t="n">
         <v>0.09120000153779984</v>
@@ -1677,10 +1677,10 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.771</v>
+        <v>0.756</v>
       </c>
       <c r="C79" t="n">
-        <v>0.392</v>
+        <v>0.35</v>
       </c>
       <c r="D79" t="n">
         <v>0.2912999987602234</v>
@@ -1693,10 +1693,10 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.922</v>
+        <v>0.916</v>
       </c>
       <c r="C80" t="n">
-        <v>0.528</v>
+        <v>0.521</v>
       </c>
       <c r="D80" t="n">
         <v>0.1342999935150146</v>
@@ -1709,10 +1709,10 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1.528</v>
+        <v>1.083</v>
       </c>
       <c r="C81" t="n">
-        <v>2.258</v>
+        <v>0.598</v>
       </c>
       <c r="D81" t="n">
         <v>0.324400007724762</v>
@@ -1725,10 +1725,10 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1.695</v>
+        <v>1.623</v>
       </c>
       <c r="C82" t="n">
-        <v>1.056</v>
+        <v>1.052</v>
       </c>
       <c r="D82" t="n">
         <v>0.135900005698204</v>
@@ -1741,10 +1741,10 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1.029</v>
+        <v>0.731</v>
       </c>
       <c r="C83" t="n">
-        <v>1.954</v>
+        <v>0.666</v>
       </c>
       <c r="D83" t="n">
         <v>0.336899995803833</v>
@@ -1757,10 +1757,10 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1.842</v>
+        <v>1.824</v>
       </c>
       <c r="C84" t="n">
-        <v>1.468</v>
+        <v>1.479</v>
       </c>
       <c r="D84" t="n">
         <v>0.1439999938011169</v>
@@ -1773,10 +1773,10 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1.401</v>
+        <v>1.346</v>
       </c>
       <c r="C85" t="n">
-        <v>0.706</v>
+        <v>0.703</v>
       </c>
       <c r="D85" t="n">
         <v>0.4137000143527985</v>
@@ -1789,10 +1789,10 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.538</v>
       </c>
       <c r="C86" t="n">
-        <v>0.479</v>
+        <v>0.395</v>
       </c>
       <c r="D86" t="n">
         <v>0.1415999978780746</v>
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="C87" t="n">
-        <v>0.578</v>
+        <v>0.577</v>
       </c>
       <c r="D87" t="n">
         <v>0.4268999993801117</v>
@@ -1821,10 +1821,10 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>2.768</v>
+        <v>2.763</v>
       </c>
       <c r="C88" t="n">
-        <v>2.449</v>
+        <v>2.452</v>
       </c>
       <c r="D88" t="n">
         <v>0.255299985408783</v>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1.129</v>
+        <v>1.127</v>
       </c>
       <c r="C89" t="n">
         <v>0.601</v>
@@ -1853,10 +1853,10 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>2.802</v>
+        <v>2.768</v>
       </c>
       <c r="C90" t="n">
-        <v>3.2</v>
+        <v>3.207</v>
       </c>
       <c r="D90" t="n">
         <v>0.2619999945163727</v>
@@ -1869,10 +1869,10 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>0.921</v>
+        <v>0.887</v>
       </c>
       <c r="C91" t="n">
-        <v>0.778</v>
+        <v>0.766</v>
       </c>
       <c r="D91" t="n">
         <v>0.2906999886035919</v>
@@ -1885,10 +1885,10 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3.877</v>
+        <v>3.887</v>
       </c>
       <c r="C92" t="n">
-        <v>8.19</v>
+        <v>8.186</v>
       </c>
       <c r="D92" t="n">
         <v>0.09570000320672989</v>
@@ -1901,10 +1901,10 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1.318</v>
+        <v>1.182</v>
       </c>
       <c r="C93" t="n">
-        <v>1.103</v>
+        <v>0.767</v>
       </c>
       <c r="D93" t="n">
         <v>0.339599996805191</v>
@@ -1917,10 +1917,10 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1.341</v>
+        <v>1.339</v>
       </c>
       <c r="C94" t="n">
-        <v>0.639</v>
+        <v>0.64</v>
       </c>
       <c r="D94" t="n">
         <v>0.3050000071525574</v>
@@ -1933,10 +1933,10 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1.083</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="C95" t="n">
-        <v>1.361</v>
+        <v>0.493</v>
       </c>
       <c r="D95" t="n">
         <v>0.3312999904155731</v>
@@ -1949,10 +1949,10 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>0.951</v>
+        <v>0.961</v>
       </c>
       <c r="C96" t="n">
-        <v>0.556</v>
+        <v>0.553</v>
       </c>
       <c r="D96" t="n">
         <v>0.0925000011920929</v>
@@ -1965,10 +1965,10 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1.181</v>
+        <v>0.798</v>
       </c>
       <c r="C97" t="n">
-        <v>1.872</v>
+        <v>0.547</v>
       </c>
       <c r="D97" t="n">
         <v>0.3023999929428101</v>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>1.641</v>
+        <v>1.503</v>
       </c>
       <c r="C98" t="n">
-        <v>0.994</v>
+        <v>0.907</v>
       </c>
       <c r="D98" t="n">
         <v>0.1427000015974045</v>
@@ -1997,10 +1997,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>0.845</v>
+        <v>0.892</v>
       </c>
       <c r="C99" t="n">
-        <v>0.782</v>
+        <v>0.826</v>
       </c>
       <c r="D99" t="n">
         <v>0.4410000145435333</v>
@@ -2013,10 +2013,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>1.568</v>
+        <v>1.515</v>
       </c>
       <c r="C100" t="n">
-        <v>0.627</v>
+        <v>0.68</v>
       </c>
       <c r="D100" t="n">
         <v>0.1524000018835068</v>
@@ -2029,10 +2029,10 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.707</v>
       </c>
       <c r="C101" t="n">
-        <v>0.406</v>
+        <v>0.409</v>
       </c>
       <c r="D101" t="n">
         <v>0.3127999901771545</v>
@@ -2045,10 +2045,10 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1.309</v>
+        <v>1.297</v>
       </c>
       <c r="C102" t="n">
-        <v>0.702</v>
+        <v>0.698</v>
       </c>
       <c r="D102" t="n">
         <v>0.3959000110626221</v>
@@ -2061,10 +2061,10 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0.908</v>
+        <v>1.924</v>
       </c>
       <c r="C103" t="n">
-        <v>1.388</v>
+        <v>5.885</v>
       </c>
       <c r="D103" t="n">
         <v>0.2267999947071075</v>
@@ -2077,10 +2077,10 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>1.644</v>
+        <v>1.601</v>
       </c>
       <c r="C104" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.591</v>
       </c>
       <c r="D104" t="n">
         <v>0.0982000008225441</v>
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.965</v>
+        <v>0.987</v>
       </c>
       <c r="C105" t="n">
-        <v>0.324</v>
+        <v>0.351</v>
       </c>
       <c r="D105" t="n">
         <v>0.4679000079631805</v>
@@ -2109,10 +2109,10 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1.359</v>
+        <v>1.366</v>
       </c>
       <c r="C106" t="n">
-        <v>0.781</v>
+        <v>0.773</v>
       </c>
       <c r="D106" t="n">
         <v>0.1008000001311302</v>
@@ -2125,10 +2125,10 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>1.074</v>
+        <v>1.067</v>
       </c>
       <c r="C107" t="n">
-        <v>0.531</v>
+        <v>0.521</v>
       </c>
       <c r="D107" t="n">
         <v>0.3774000108242035</v>
@@ -2141,10 +2141,10 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>1.278</v>
+        <v>1.271</v>
       </c>
       <c r="C108" t="n">
-        <v>1.147</v>
+        <v>1.143</v>
       </c>
       <c r="D108" t="n">
         <v>0.3086000084877014</v>
@@ -2157,10 +2157,10 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>1.993</v>
+        <v>2.016</v>
       </c>
       <c r="C109" t="n">
-        <v>1.522</v>
+        <v>1.504</v>
       </c>
       <c r="D109" t="n">
         <v>0.4546999931335449</v>
@@ -2173,10 +2173,10 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>1.445</v>
+        <v>1.448</v>
       </c>
       <c r="C110" t="n">
-        <v>0.621</v>
+        <v>0.625</v>
       </c>
       <c r="D110" t="n">
         <v>0.1004000008106232</v>
@@ -2189,10 +2189,10 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>1.03</v>
+        <v>0.968</v>
       </c>
       <c r="C111" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="D111" t="n">
         <v>0.3540999889373779</v>
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1.086</v>
+        <v>1.088</v>
       </c>
       <c r="C112" t="n">
         <v>0.774</v>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.819</v>
+        <v>0.8</v>
       </c>
       <c r="C113" t="n">
-        <v>0.489</v>
+        <v>0.457</v>
       </c>
       <c r="D113" t="n">
         <v>0.1560000032186508</v>
@@ -2237,10 +2237,10 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>2.057</v>
+        <v>1.844</v>
       </c>
       <c r="C114" t="n">
-        <v>1.269</v>
+        <v>0.823</v>
       </c>
       <c r="D114" t="n">
         <v>0.2572000026702881</v>
@@ -2253,10 +2253,10 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.986</v>
+        <v>0.928</v>
       </c>
       <c r="C115" t="n">
-        <v>0.725</v>
+        <v>0.716</v>
       </c>
       <c r="D115" t="n">
         <v>0.3124000132083893</v>
@@ -2269,10 +2269,10 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1.209</v>
+        <v>1.215</v>
       </c>
       <c r="C116" t="n">
-        <v>0.663</v>
+        <v>0.657</v>
       </c>
       <c r="D116" t="n">
         <v>0.09830000251531601</v>
@@ -2285,10 +2285,10 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>0.901</v>
+        <v>0.884</v>
       </c>
       <c r="C117" t="n">
-        <v>0.431</v>
+        <v>0.395</v>
       </c>
       <c r="D117" t="n">
         <v>0.3357000052928925</v>
@@ -2301,10 +2301,10 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>0.944</v>
+        <v>1.042</v>
       </c>
       <c r="C118" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.851</v>
       </c>
       <c r="D118" t="n">
         <v>0.09309999644756317</v>
@@ -2317,10 +2317,10 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>0.991</v>
+        <v>0.978</v>
       </c>
       <c r="C119" t="n">
-        <v>1.397</v>
+        <v>1.342</v>
       </c>
       <c r="D119" t="n">
         <v>0.3041000068187714</v>
@@ -2333,10 +2333,10 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>1.474</v>
+        <v>1.464</v>
       </c>
       <c r="C120" t="n">
-        <v>1.873</v>
+        <v>1.83</v>
       </c>
       <c r="D120" t="n">
         <v>0.09640000015497208</v>
@@ -2349,10 +2349,10 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>1.183</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="C121" t="n">
-        <v>2.39</v>
+        <v>0.489</v>
       </c>
       <c r="D121" t="n">
         <v>0.3061999976634979</v>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>1.297</v>
+        <v>1.307</v>
       </c>
       <c r="C122" t="n">
         <v>0.632</v>
@@ -2381,10 +2381,10 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1.16</v>
+        <v>1.176</v>
       </c>
       <c r="C123" t="n">
-        <v>0.477</v>
+        <v>0.476</v>
       </c>
       <c r="D123" t="n">
         <v>0.3278000056743622</v>
@@ -2397,10 +2397,10 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>1.325</v>
+        <v>1.339</v>
       </c>
       <c r="C124" t="n">
-        <v>0.586</v>
+        <v>0.6</v>
       </c>
       <c r="D124" t="n">
         <v>0.29789999127388</v>
@@ -2413,10 +2413,10 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1.068</v>
+        <v>0.763</v>
       </c>
       <c r="C125" t="n">
-        <v>1.763</v>
+        <v>0.539</v>
       </c>
       <c r="D125" t="n">
         <v>0.324400007724762</v>
@@ -2429,10 +2429,10 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>2.139</v>
+        <v>2.132</v>
       </c>
       <c r="C126" t="n">
-        <v>0.915</v>
+        <v>0.917</v>
       </c>
       <c r="D126" t="n">
         <v>0.3260000050067902</v>
@@ -2445,10 +2445,10 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2.022</v>
+        <v>1.987</v>
       </c>
       <c r="C127" t="n">
-        <v>1.587</v>
+        <v>1.497</v>
       </c>
       <c r="D127" t="n">
         <v>0.7678999900817871</v>
@@ -2461,10 +2461,10 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.949</v>
+        <v>0.846</v>
       </c>
       <c r="C128" t="n">
-        <v>0.712</v>
+        <v>0.643</v>
       </c>
       <c r="D128" t="n">
         <v>0.0885000005364418</v>
@@ -2477,10 +2477,10 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="C129" t="n">
-        <v>0.486</v>
+        <v>0.487</v>
       </c>
       <c r="D129" t="n">
         <v>0.42289999127388</v>
@@ -2493,10 +2493,10 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.927</v>
+        <v>0.949</v>
       </c>
       <c r="C130" t="n">
-        <v>0.474</v>
+        <v>0.473</v>
       </c>
       <c r="D130" t="n">
         <v>0.1381999999284744</v>
@@ -2509,10 +2509,10 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0.705</v>
+        <v>0.67</v>
       </c>
       <c r="C131" t="n">
-        <v>0.361</v>
+        <v>0.309</v>
       </c>
       <c r="D131" t="n">
         <v>0.3075999915599823</v>
@@ -2525,10 +2525,10 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>1.187</v>
+        <v>1.157</v>
       </c>
       <c r="C132" t="n">
-        <v>0.709</v>
+        <v>0.712</v>
       </c>
       <c r="D132" t="n">
         <v>0.1013000011444092</v>
@@ -2541,10 +2541,10 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>0.55</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="C133" t="n">
-        <v>0.302</v>
+        <v>0.327</v>
       </c>
       <c r="D133" t="n">
         <v>0.4133000075817108</v>
@@ -2557,10 +2557,10 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0.695</v>
+        <v>0.677</v>
       </c>
       <c r="C134" t="n">
-        <v>0.333</v>
+        <v>0.351</v>
       </c>
       <c r="D134" t="n">
         <v>0.2603000104427338</v>
@@ -2573,10 +2573,10 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>0.981</v>
+        <v>0.928</v>
       </c>
       <c r="C135" t="n">
-        <v>0.623</v>
+        <v>0.619</v>
       </c>
       <c r="D135" t="n">
         <v>0.1673000007867813</v>
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1.64</v>
+        <v>1.666</v>
       </c>
       <c r="C136" t="n">
-        <v>1.18</v>
+        <v>1.152</v>
       </c>
       <c r="D136" t="n">
         <v>0.3792999982833862</v>
@@ -2605,10 +2605,10 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1.004</v>
+        <v>0.747</v>
       </c>
       <c r="C137" t="n">
-        <v>1.717</v>
+        <v>0.635</v>
       </c>
       <c r="D137" t="n">
         <v>0.4336000084877014</v>
@@ -2621,10 +2621,10 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>1.209</v>
+        <v>1.192</v>
       </c>
       <c r="C138" t="n">
-        <v>0.608</v>
+        <v>0.622</v>
       </c>
       <c r="D138" t="n">
         <v>0.4079999923706055</v>
@@ -2637,10 +2637,10 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>1.861</v>
+        <v>1.851</v>
       </c>
       <c r="C139" t="n">
-        <v>1.382</v>
+        <v>1.388</v>
       </c>
       <c r="D139" t="n">
         <v>0.3330000042915344</v>
@@ -2653,10 +2653,10 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1.953</v>
+        <v>1.982</v>
       </c>
       <c r="C140" t="n">
-        <v>1.027</v>
+        <v>0.993</v>
       </c>
       <c r="D140" t="n">
         <v>0.1648000031709671</v>
@@ -2669,10 +2669,10 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1.227</v>
+        <v>1.178</v>
       </c>
       <c r="C141" t="n">
-        <v>0.492</v>
+        <v>0.45</v>
       </c>
       <c r="D141" t="n">
         <v>0.3513999879360199</v>
@@ -2685,10 +2685,10 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>3.369</v>
+        <v>3.254</v>
       </c>
       <c r="C142" t="n">
-        <v>2.86</v>
+        <v>2.919</v>
       </c>
       <c r="D142" t="n">
         <v>0.3463000059127808</v>
@@ -2701,10 +2701,10 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>2.889</v>
+        <v>2.878</v>
       </c>
       <c r="C143" t="n">
-        <v>3.363</v>
+        <v>3.368</v>
       </c>
       <c r="D143" t="n">
         <v>0.1383000016212463</v>
@@ -2717,10 +2717,10 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>1.16</v>
+        <v>1.166</v>
       </c>
       <c r="C144" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.698</v>
       </c>
       <c r="D144" t="n">
         <v>0.1001999974250793</v>
@@ -2733,10 +2733,10 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1.175</v>
+        <v>1.171</v>
       </c>
       <c r="C145" t="n">
-        <v>0.728</v>
+        <v>0.73</v>
       </c>
       <c r="D145" t="n">
         <v>0.414000004529953</v>
@@ -2749,10 +2749,10 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1.222</v>
+        <v>1.175</v>
       </c>
       <c r="C146" t="n">
-        <v>0.483</v>
+        <v>0.495</v>
       </c>
       <c r="D146" t="n">
         <v>0.1403000056743622</v>
@@ -2765,10 +2765,10 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>0.844</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="C147" t="n">
-        <v>0.267</v>
+        <v>0.492</v>
       </c>
       <c r="D147" t="n">
         <v>0.3131999969482422</v>
@@ -2781,10 +2781,10 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0.949</v>
+        <v>0.925</v>
       </c>
       <c r="C148" t="n">
-        <v>0.4</v>
+        <v>0.386</v>
       </c>
       <c r="D148" t="n">
         <v>0.3167000114917755</v>
@@ -2797,10 +2797,10 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>1.08</v>
+        <v>1.091</v>
       </c>
       <c r="C149" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.679</v>
       </c>
       <c r="D149" t="n">
         <v>0.3939999938011169</v>
@@ -2813,10 +2813,10 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1.834</v>
+        <v>1.797</v>
       </c>
       <c r="C150" t="n">
-        <v>0.903</v>
+        <v>0.909</v>
       </c>
       <c r="D150" t="n">
         <v>0.09690000116825104</v>
@@ -2829,10 +2829,10 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>0.755</v>
+        <v>0.748</v>
       </c>
       <c r="C151" t="n">
-        <v>0.404</v>
+        <v>0.403</v>
       </c>
       <c r="D151" t="n">
         <v>0.2870999872684479</v>
@@ -2845,10 +2845,10 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>3.148</v>
+        <v>3.372</v>
       </c>
       <c r="C152" t="n">
-        <v>2.526</v>
+        <v>3.032</v>
       </c>
       <c r="D152" t="n">
         <v>0.2554999887943268</v>
@@ -2861,10 +2861,10 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.945</v>
       </c>
       <c r="C153" t="n">
-        <v>0.379</v>
+        <v>0.762</v>
       </c>
       <c r="D153" t="n">
         <v>0.4997000098228455</v>
@@ -2877,10 +2877,10 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>2.409</v>
+        <v>1.996</v>
       </c>
       <c r="C154" t="n">
-        <v>2.109</v>
+        <v>1.264</v>
       </c>
       <c r="D154" t="n">
         <v>0.2380000054836273</v>
@@ -2893,10 +2893,10 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>0.833</v>
+        <v>0.894</v>
       </c>
       <c r="C155" t="n">
-        <v>0.275</v>
+        <v>0.377</v>
       </c>
       <c r="D155" t="n">
         <v>0.3458999991416931</v>
@@ -2909,10 +2909,10 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>1.08</v>
+        <v>1.078</v>
       </c>
       <c r="C156" t="n">
-        <v>0.64</v>
+        <v>0.641</v>
       </c>
       <c r="D156" t="n">
         <v>0.2102999985218048</v>
@@ -2925,10 +2925,10 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>0.766</v>
+        <v>0.637</v>
       </c>
       <c r="C157" t="n">
-        <v>0.837</v>
+        <v>0.432</v>
       </c>
       <c r="D157" t="n">
         <v>0.160400003194809</v>
@@ -2941,10 +2941,10 @@
         </is>
       </c>
       <c r="B158" t="n">
-        <v>0.865</v>
+        <v>0.842</v>
       </c>
       <c r="C158" t="n">
-        <v>0.533</v>
+        <v>0.477</v>
       </c>
       <c r="D158" t="n">
         <v>0.09160000085830688</v>
@@ -2957,10 +2957,10 @@
         </is>
       </c>
       <c r="B159" t="n">
-        <v>0.601</v>
+        <v>0.58</v>
       </c>
       <c r="C159" t="n">
-        <v>0.412</v>
+        <v>0.421</v>
       </c>
       <c r="D159" t="n">
         <v>0.3632000088691711</v>
@@ -2973,10 +2973,10 @@
         </is>
       </c>
       <c r="B160" t="n">
-        <v>1.689</v>
+        <v>1.705</v>
       </c>
       <c r="C160" t="n">
-        <v>1.176</v>
+        <v>1.162</v>
       </c>
       <c r="D160" t="n">
         <v>0.1358000040054321</v>
@@ -2989,10 +2989,10 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0.783</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="C161" t="n">
-        <v>0.403</v>
+        <v>0.423</v>
       </c>
       <c r="D161" t="n">
         <v>0.3492000102996826</v>
@@ -3005,10 +3005,10 @@
         </is>
       </c>
       <c r="B162" t="n">
-        <v>1.477</v>
+        <v>1.478</v>
       </c>
       <c r="C162" t="n">
-        <v>0.669</v>
+        <v>0.67</v>
       </c>
       <c r="D162" t="n">
         <v>0.1501999944448471</v>
@@ -3021,10 +3021,10 @@
         </is>
       </c>
       <c r="B163" t="n">
-        <v>1.448</v>
+        <v>1.488</v>
       </c>
       <c r="C163" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="D163" t="n">
         <v>0.371399998664856</v>
@@ -3037,10 +3037,10 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>1.469</v>
+        <v>1.406</v>
       </c>
       <c r="C164" t="n">
-        <v>0.989</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="D164" t="n">
         <v>0.3899999856948853</v>
@@ -3053,10 +3053,10 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>0.844</v>
+        <v>0.856</v>
       </c>
       <c r="C165" t="n">
-        <v>0.646</v>
+        <v>0.656</v>
       </c>
       <c r="D165" t="n">
         <v>0.2442999929189682</v>
@@ -3069,10 +3069,10 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>1.596</v>
+        <v>1.508</v>
       </c>
       <c r="C166" t="n">
-        <v>1.308</v>
+        <v>1.32</v>
       </c>
       <c r="D166" t="n">
         <v>0.3084000051021576</v>
@@ -3085,10 +3085,10 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>0.909</v>
+        <v>0.84</v>
       </c>
       <c r="C167" t="n">
-        <v>0.585</v>
+        <v>0.392</v>
       </c>
       <c r="D167" t="n">
         <v>0.6453999876976013</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>0.983</v>
+        <v>0.979</v>
       </c>
       <c r="C168" t="n">
         <v>0.359</v>
@@ -3117,10 +3117,10 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.842</v>
       </c>
       <c r="C169" t="n">
-        <v>0.549</v>
+        <v>0.546</v>
       </c>
       <c r="D169" t="n">
         <v>0.1394000053405762</v>
@@ -3133,10 +3133,10 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>1.048</v>
+        <v>1.022</v>
       </c>
       <c r="C170" t="n">
-        <v>0.473</v>
+        <v>0.487</v>
       </c>
       <c r="D170" t="n">
         <v>0.09920000284910202</v>
@@ -3149,10 +3149,10 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>1.36</v>
+        <v>1.241</v>
       </c>
       <c r="C171" t="n">
-        <v>0.623</v>
+        <v>0.438</v>
       </c>
       <c r="D171" t="n">
         <v>0.163100004196167</v>
@@ -3165,10 +3165,10 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.929</v>
       </c>
       <c r="C172" t="n">
-        <v>0.507</v>
+        <v>0.51</v>
       </c>
       <c r="D172" t="n">
         <v>0.101000003516674</v>
@@ -3181,10 +3181,10 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="C173" t="n">
-        <v>0.406</v>
+        <v>0.41</v>
       </c>
       <c r="D173" t="n">
         <v>0.4025000035762787</v>
@@ -3197,10 +3197,10 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.999</v>
       </c>
       <c r="C174" t="n">
-        <v>0.678</v>
+        <v>0.719</v>
       </c>
       <c r="D174" t="n">
         <v>0.09549999982118607</v>
@@ -3213,10 +3213,10 @@
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0.739</v>
+        <v>0.715</v>
       </c>
       <c r="C175" t="n">
-        <v>0.467</v>
+        <v>0.429</v>
       </c>
       <c r="D175" t="n">
         <v>0.3379999995231628</v>
@@ -3229,10 +3229,10 @@
         </is>
       </c>
       <c r="B176" t="n">
-        <v>1.108</v>
+        <v>1.081</v>
       </c>
       <c r="C176" t="n">
-        <v>0.484</v>
+        <v>0.48</v>
       </c>
       <c r="D176" t="n">
         <v>0.08709999918937683</v>
@@ -3245,10 +3245,10 @@
         </is>
       </c>
       <c r="B177" t="n">
-        <v>2.502</v>
+        <v>2.669</v>
       </c>
       <c r="C177" t="n">
-        <v>2.903</v>
+        <v>3.406</v>
       </c>
       <c r="D177" t="n">
         <v>0.1474999934434891</v>
@@ -3261,10 +3261,10 @@
         </is>
       </c>
       <c r="B178" t="n">
-        <v>1.078</v>
+        <v>1.101</v>
       </c>
       <c r="C178" t="n">
-        <v>0.514</v>
+        <v>0.533</v>
       </c>
       <c r="D178" t="n">
         <v>0.2019000053405762</v>
@@ -3277,10 +3277,10 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>0.896</v>
+        <v>0.908</v>
       </c>
       <c r="C179" t="n">
-        <v>0.723</v>
+        <v>0.726</v>
       </c>
       <c r="D179" t="n">
         <v>0.1916999965906143</v>

</xml_diff>